<commit_message>
Update requirements to allow for newer package versions
</commit_message>
<xml_diff>
--- a/registros.xlsx
+++ b/registros.xlsx
@@ -26,16 +26,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,7 +43,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -54,21 +51,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -443,17 +431,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Cedula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Nombre</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Telefono</t>
         </is>
@@ -491,12 +479,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Rol</t>
         </is>
@@ -557,42 +545,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Referencia</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Codigo de barras</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Precio de adquisicion</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Precio venta</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Unidades actuales</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Producto disponible</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
@@ -649,12 +637,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Metodo de pago</t>
         </is>
@@ -715,42 +703,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ID venta</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Cedula</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Producto</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>ID_MetodoPago</t>
         </is>
@@ -969,10 +957,8 @@
       <c r="A8" t="n">
         <v>409</v>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>71722939</t>
-        </is>
+      <c r="B8" t="n">
+        <v>71722939</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -991,10 +977,8 @@
           <t>06/06/2024 15:23</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="F8" t="n">
+        <v>3</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1010,10 +994,8 @@
       <c r="A9" t="n">
         <v>0</v>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>71722939</t>
-        </is>
+      <c r="B9" t="n">
+        <v>71722939</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1031,10 +1013,8 @@
           <t>06/06/2024 15:23</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="F9" t="n">
+        <v>3</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1071,42 +1051,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ID venta</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Cedula</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cliente</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Servicio</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>ID_MetodoPago</t>
         </is>
@@ -1132,17 +1112,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ID servicio</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Nombre Servicio</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Costo</t>
         </is>
@@ -1183,27 +1163,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ID Reserva</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Cliente</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Servicio</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Fecha Reserva</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fecha Servicio</t>
         </is>
@@ -1233,37 +1213,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Cedula</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Cliente</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>SubtotalProductos</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>SubtotalServicios</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Metodo de pago</t>
         </is>
@@ -1290,22 +1270,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ID usuario</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>usuario</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>contraseña</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Rol ID</t>
         </is>

</xml_diff>